<commit_message>
feat: add axis name 'Axe 1 : Etat des lieux quantitatif du Startup Act' to charte and plan de veille (MD/PDF/XLSX)
</commit_message>
<xml_diff>
--- a/livrables/2_plan_de_veille_AE1_etat_des_lieux_quantitatif.xlsx
+++ b/livrables/2_plan_de_veille_AE1_etat_des_lieux_quantitatif.xlsx
@@ -14,7 +14,10 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="59" uniqueCount="58">
+  <si>
+    <t>Axe 1 : État des lieux quantitatif du Startup Act</t>
+  </si>
   <si>
     <t>Plan de veille AE1 — État des lieux quantitatif</t>
   </si>
@@ -582,7 +585,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.7109375" customWidth="1"/>
@@ -615,194 +618,206 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="4" spans="1:7" ht="28" customHeight="1">
-      <c r="A4" s="3" t="s">
+    <row r="3" spans="1:7">
+      <c r="A3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="5" spans="1:7" ht="28" customHeight="1">
+      <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C4" s="3" t="s">
+      <c r="B5" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="G4" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:7">
-      <c r="A5" s="4" t="s">
+      <c r="G5" s="3" t="s">
         <v>9</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="G5" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>12</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="G6" s="5" t="s">
         <v>16</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G6" s="5" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="G7" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="5" t="s">
+        <v>29</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>30</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>33</v>
-      </c>
-      <c r="E8" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="F8" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="G8" s="5" t="s">
-        <v>36</v>
       </c>
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="5" t="s">
         <v>37</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>40</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>42</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:7">
       <c r="A10" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>43</v>
+      </c>
+      <c r="G10" s="5" t="s">
         <v>44</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="G10" s="5" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="11" spans="1:7">
       <c r="A11" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>46</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="F11" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="G11" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7">
+      <c r="A12" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="B12" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="C12" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="D12" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="F11" s="5" t="s">
+      <c r="E12" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="G11" s="5" t="s">
+      <c r="F12" s="5" t="s">
         <v>56</v>
       </c>
+      <c r="G12" s="5" t="s">
+        <v>57</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:G3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>